<commit_message>
midterm scheduling implemented. TODO: have a constraint for off_timetable slots
</commit_message>
<xml_diff>
--- a/data/New Microsoft Excel Worksheet.xlsx
+++ b/data/New Microsoft Excel Worksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B795BBC-29DB-4232-997E-53A36DCE9072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BE2888-D9BC-4A4C-80B8-840BAE8152C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="5940" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -399,39 +399,21 @@
     <t>MÜH. D-E BLOK-K2-1-DERSLİK</t>
   </si>
   <si>
-    <t>D-201</t>
-  </si>
-  <si>
     <t>MÜH. D-E BLOK-K2-2-DERSLİK</t>
   </si>
   <si>
-    <t>D-202</t>
-  </si>
-  <si>
     <t>MÜH. D-E BLOK-K2-3-DERSLİK</t>
   </si>
   <si>
-    <t>D-203</t>
-  </si>
-  <si>
     <t>MÜH. D-E BLOK-K2-7-DERSLİK</t>
   </si>
   <si>
-    <t>D-204</t>
-  </si>
-  <si>
     <t>MÜH. D-E BLOK-K2-8-DERSLİK</t>
   </si>
   <si>
-    <t>D-205</t>
-  </si>
-  <si>
     <t>MÜH. D-E BLOK-K2-9-DERSLİK</t>
   </si>
   <si>
-    <t>D-206</t>
-  </si>
-  <si>
     <t>ES-K3-13</t>
   </si>
   <si>
@@ -531,75 +513,15 @@
     <t>SERİK</t>
   </si>
   <si>
-    <t>Ylab-2</t>
-  </si>
-  <si>
     <t>BZ01</t>
   </si>
   <si>
-    <t>Ylab-1</t>
-  </si>
-  <si>
-    <t>CAD</t>
-  </si>
-  <si>
-    <t>Amfi03</t>
-  </si>
-  <si>
-    <t>Amfi04</t>
-  </si>
-  <si>
-    <t>C-209</t>
-  </si>
-  <si>
-    <t>C-210</t>
-  </si>
-  <si>
-    <t>C-211</t>
-  </si>
-  <si>
-    <t>C-208</t>
-  </si>
-  <si>
-    <t>C-207</t>
-  </si>
-  <si>
-    <t>C-206</t>
-  </si>
-  <si>
-    <t>C-205</t>
-  </si>
-  <si>
-    <t>C-204</t>
-  </si>
-  <si>
-    <t>C-203</t>
-  </si>
-  <si>
-    <t>C-202</t>
-  </si>
-  <si>
-    <t>C-201</t>
-  </si>
-  <si>
-    <t>B-102</t>
-  </si>
-  <si>
     <t>DZ01</t>
   </si>
   <si>
-    <t>C-212</t>
-  </si>
-  <si>
-    <t>C-213</t>
-  </si>
-  <si>
     <t>BB04</t>
   </si>
   <si>
-    <t>Ylab-3</t>
-  </si>
-  <si>
     <t>Capacity</t>
   </si>
   <si>
@@ -610,6 +532,84 @@
   </si>
   <si>
     <t>Lab</t>
+  </si>
+  <si>
+    <t>YLAB 2</t>
+  </si>
+  <si>
+    <t>C201</t>
+  </si>
+  <si>
+    <t>C202</t>
+  </si>
+  <si>
+    <t>C203</t>
+  </si>
+  <si>
+    <t>C204</t>
+  </si>
+  <si>
+    <t>C212</t>
+  </si>
+  <si>
+    <t>C205</t>
+  </si>
+  <si>
+    <t>C206</t>
+  </si>
+  <si>
+    <t>C207</t>
+  </si>
+  <si>
+    <t>C208</t>
+  </si>
+  <si>
+    <t>C213</t>
+  </si>
+  <si>
+    <t>C209</t>
+  </si>
+  <si>
+    <t>C210</t>
+  </si>
+  <si>
+    <t>C211</t>
+  </si>
+  <si>
+    <t>Amfi 4</t>
+  </si>
+  <si>
+    <t>Amfi 3</t>
+  </si>
+  <si>
+    <t>YLAB 1</t>
+  </si>
+  <si>
+    <t>B102</t>
+  </si>
+  <si>
+    <t>CAD1</t>
+  </si>
+  <si>
+    <t>YLAB 3</t>
+  </si>
+  <si>
+    <t>D201</t>
+  </si>
+  <si>
+    <t>D202</t>
+  </si>
+  <si>
+    <t>D203</t>
+  </si>
+  <si>
+    <t>D204</t>
+  </si>
+  <si>
+    <t>D205</t>
+  </si>
+  <si>
+    <t>D206</t>
   </si>
 </sst>
 </file>
@@ -882,18 +882,6 @@
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
@@ -907,27 +895,19 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -952,6 +932,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1243,15 +1243,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="26" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="27"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="24"/>
       <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1259,10 +1259,10 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>4</v>
@@ -1271,7 +1271,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>6</v>
@@ -1282,32 +1282,32 @@
       <c r="O1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="29" t="s">
+      <c r="P1" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="27"/>
+      <c r="Q1" s="34"/>
+      <c r="R1" s="24"/>
       <c r="S1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="29" t="s">
+      <c r="T1" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="27"/>
+      <c r="U1" s="24"/>
       <c r="V1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="20" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="21"/>
-      <c r="E2" s="22"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="26"/>
       <c r="F2" s="4" t="s">
         <v>66</v>
       </c>
@@ -1336,28 +1336,28 @@
       <c r="O2" s="7">
         <v>11.25</v>
       </c>
-      <c r="P2" s="30">
+      <c r="P2" s="33">
         <v>16</v>
       </c>
-      <c r="Q2" s="28"/>
-      <c r="R2" s="27"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="24"/>
       <c r="S2" s="7">
         <v>2.98</v>
       </c>
-      <c r="T2" s="30">
+      <c r="T2" s="33">
         <v>536.4</v>
       </c>
-      <c r="U2" s="27"/>
+      <c r="U2" s="24"/>
       <c r="V2" s="7">
         <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="23"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="22"/>
       <c r="F3" s="4" t="s">
         <v>68</v>
       </c>
@@ -1386,28 +1386,28 @@
       <c r="O3" s="7">
         <v>11.25</v>
       </c>
-      <c r="P3" s="30">
+      <c r="P3" s="33">
         <v>16</v>
       </c>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="27"/>
+      <c r="Q3" s="34"/>
+      <c r="R3" s="24"/>
       <c r="S3" s="7">
         <v>2.98</v>
       </c>
-      <c r="T3" s="30">
+      <c r="T3" s="33">
         <v>536.4</v>
       </c>
-      <c r="U3" s="27"/>
+      <c r="U3" s="24"/>
       <c r="V3" s="7">
         <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="52.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="23"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="25"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="22"/>
       <c r="F4" s="4" t="s">
         <v>35</v>
       </c>
@@ -1436,28 +1436,28 @@
       <c r="O4" s="7">
         <v>14.86</v>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="33">
         <v>6.93</v>
       </c>
-      <c r="Q4" s="28"/>
-      <c r="R4" s="27"/>
+      <c r="Q4" s="34"/>
+      <c r="R4" s="24"/>
       <c r="S4" s="7">
         <v>3.37</v>
       </c>
-      <c r="T4" s="30">
+      <c r="T4" s="33">
         <v>347.04199999999997</v>
       </c>
-      <c r="U4" s="27"/>
+      <c r="U4" s="24"/>
       <c r="V4" s="7">
         <v>102.98</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A5" s="23"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="22"/>
       <c r="F5" s="4" t="s">
         <v>71</v>
       </c>
@@ -1465,10 +1465,10 @@
         <v>72</v>
       </c>
       <c r="H5" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>160</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>29</v>
@@ -1488,28 +1488,28 @@
       <c r="O5" s="7">
         <v>18.46</v>
       </c>
-      <c r="P5" s="30">
+      <c r="P5" s="33">
         <v>6.9</v>
       </c>
-      <c r="Q5" s="28"/>
-      <c r="R5" s="27"/>
+      <c r="Q5" s="34"/>
+      <c r="R5" s="24"/>
       <c r="S5" s="7">
         <v>2.91</v>
       </c>
-      <c r="T5" s="30">
+      <c r="T5" s="33">
         <v>370.65800000000002</v>
       </c>
-      <c r="U5" s="27"/>
+      <c r="U5" s="24"/>
       <c r="V5" s="7">
         <v>127.374</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A6" s="23"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="22"/>
       <c r="F6" s="4" t="s">
         <v>73</v>
       </c>
@@ -1538,28 +1538,28 @@
       <c r="O6" s="7">
         <v>18.079999999999998</v>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="33">
         <v>6.91</v>
       </c>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="27"/>
+      <c r="Q6" s="34"/>
+      <c r="R6" s="24"/>
       <c r="S6" s="7">
         <v>2.89</v>
       </c>
-      <c r="T6" s="30">
+      <c r="T6" s="33">
         <v>361.05599999999998</v>
       </c>
-      <c r="U6" s="27"/>
+      <c r="U6" s="24"/>
       <c r="V6" s="7">
         <v>124.93300000000001</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A7" s="23"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="22"/>
       <c r="F7" s="4" t="s">
         <v>75</v>
       </c>
@@ -1588,28 +1588,28 @@
       <c r="O7" s="7">
         <v>17.88</v>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="33">
         <v>6.75</v>
       </c>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="27"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="24"/>
       <c r="S7" s="7">
         <v>2.9</v>
       </c>
-      <c r="T7" s="30">
+      <c r="T7" s="33">
         <v>350.00099999999998</v>
       </c>
-      <c r="U7" s="27"/>
+      <c r="U7" s="24"/>
       <c r="V7" s="7">
         <v>120.69</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A8" s="23"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="22"/>
       <c r="F8" s="4" t="s">
         <v>30</v>
       </c>
@@ -1638,28 +1638,28 @@
       <c r="O8" s="7">
         <v>14.93</v>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="33">
         <v>6.73</v>
       </c>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="27"/>
+      <c r="Q8" s="34"/>
+      <c r="R8" s="24"/>
       <c r="S8" s="7">
         <v>2.95</v>
       </c>
-      <c r="T8" s="30">
+      <c r="T8" s="33">
         <v>296.41300000000001</v>
       </c>
-      <c r="U8" s="27"/>
+      <c r="U8" s="24"/>
       <c r="V8" s="7">
         <v>100.479</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A9" s="23"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="25"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="22"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1688,28 +1688,28 @@
       <c r="O9" s="7">
         <v>6.7</v>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="33">
         <v>10.95</v>
       </c>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="27"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="24"/>
       <c r="S9" s="7">
         <v>2.95</v>
       </c>
-      <c r="T9" s="30">
+      <c r="T9" s="33">
         <v>216.42699999999999</v>
       </c>
-      <c r="U9" s="27"/>
+      <c r="U9" s="24"/>
       <c r="V9" s="7">
         <v>73.364999999999995</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="23"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="22"/>
       <c r="F10" s="4" t="s">
         <v>51</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>79</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>14</v>
@@ -1740,28 +1740,28 @@
       <c r="O10" s="7">
         <v>6.7</v>
       </c>
-      <c r="P10" s="30">
+      <c r="P10" s="33">
         <v>7.3</v>
       </c>
-      <c r="Q10" s="28"/>
-      <c r="R10" s="27"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="24"/>
       <c r="S10" s="7">
         <v>2.9</v>
       </c>
-      <c r="T10" s="30">
+      <c r="T10" s="33">
         <v>141.839</v>
       </c>
-      <c r="U10" s="27"/>
+      <c r="U10" s="24"/>
       <c r="V10" s="7">
         <v>48.91</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="23"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="25"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="22"/>
       <c r="F11" s="4" t="s">
         <v>59</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>80</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>14</v>
@@ -1792,28 +1792,28 @@
       <c r="O11" s="7">
         <v>10.95</v>
       </c>
-      <c r="P11" s="30">
+      <c r="P11" s="33">
         <v>6.7</v>
       </c>
-      <c r="Q11" s="28"/>
-      <c r="R11" s="27"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="24"/>
       <c r="S11" s="7">
         <v>2.9</v>
       </c>
-      <c r="T11" s="30">
+      <c r="T11" s="33">
         <v>212.75899999999999</v>
       </c>
-      <c r="U11" s="27"/>
+      <c r="U11" s="24"/>
       <c r="V11" s="7">
         <v>73.364999999999995</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="23"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="25"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="22"/>
       <c r="F12" s="4" t="s">
         <v>26</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>81</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>14</v>
@@ -1844,28 +1844,28 @@
       <c r="O12" s="7">
         <v>10.95</v>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="33">
         <v>6.75</v>
       </c>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="27"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="24"/>
       <c r="S12" s="7">
         <v>2.9</v>
       </c>
-      <c r="T12" s="30">
+      <c r="T12" s="33">
         <v>214.346</v>
       </c>
-      <c r="U12" s="27"/>
+      <c r="U12" s="24"/>
       <c r="V12" s="7">
         <v>73.912999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="23"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4" t="s">
         <v>52</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>82</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>14</v>
@@ -1896,28 +1896,28 @@
       <c r="O13" s="7">
         <v>10.25</v>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="33">
         <v>6.7</v>
       </c>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="27"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="24"/>
       <c r="S13" s="7">
         <v>2.9</v>
       </c>
-      <c r="T13" s="30">
+      <c r="T13" s="33">
         <v>199.15799999999999</v>
       </c>
-      <c r="U13" s="27"/>
+      <c r="U13" s="24"/>
       <c r="V13" s="7">
         <v>68.674999999999997</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A14" s="23"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4" t="s">
         <v>83</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>84</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>14</v>
@@ -1948,28 +1948,28 @@
       <c r="O14" s="7">
         <v>7.25</v>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="33">
         <v>7.25</v>
       </c>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="27"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="24"/>
       <c r="S14" s="7">
         <v>2.9</v>
       </c>
-      <c r="T14" s="30">
+      <c r="T14" s="33">
         <v>152.43100000000001</v>
       </c>
-      <c r="U14" s="27"/>
+      <c r="U14" s="24"/>
       <c r="V14" s="7">
         <v>52.563000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="23"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4" t="s">
         <v>42</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>85</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>14</v>
@@ -2000,28 +2000,28 @@
       <c r="O15" s="7">
         <v>6.7</v>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="33">
         <v>10.25</v>
       </c>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="27"/>
+      <c r="Q15" s="34"/>
+      <c r="R15" s="24"/>
       <c r="S15" s="7">
         <v>2.9</v>
       </c>
-      <c r="T15" s="30">
+      <c r="T15" s="33">
         <v>199.15799999999999</v>
       </c>
-      <c r="U15" s="27"/>
+      <c r="U15" s="24"/>
       <c r="V15" s="7">
         <v>68.674999999999997</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="23"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="22"/>
       <c r="F16" s="4" t="s">
         <v>43</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>86</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>14</v>
@@ -2052,28 +2052,28 @@
       <c r="O16" s="7">
         <v>6.7</v>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="33">
         <v>12.85</v>
       </c>
-      <c r="Q16" s="28"/>
-      <c r="R16" s="27"/>
+      <c r="Q16" s="34"/>
+      <c r="R16" s="24"/>
       <c r="S16" s="7">
         <v>2.9</v>
       </c>
-      <c r="T16" s="30">
+      <c r="T16" s="33">
         <v>249.67599999999999</v>
       </c>
-      <c r="U16" s="27"/>
+      <c r="U16" s="24"/>
       <c r="V16" s="7">
         <v>86.094999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="23"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="4" t="s">
         <v>57</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>87</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>14</v>
@@ -2104,28 +2104,28 @@
       <c r="O17" s="7">
         <v>6.7</v>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="33">
         <v>11.05</v>
       </c>
-      <c r="Q17" s="28"/>
-      <c r="R17" s="27"/>
+      <c r="Q17" s="34"/>
+      <c r="R17" s="24"/>
       <c r="S17" s="7">
         <v>2.9</v>
       </c>
-      <c r="T17" s="30">
+      <c r="T17" s="33">
         <v>214.702</v>
       </c>
-      <c r="U17" s="27"/>
+      <c r="U17" s="24"/>
       <c r="V17" s="7">
         <v>74.034999999999997</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="23"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="22"/>
       <c r="F18" s="4" t="s">
         <v>31</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>88</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>14</v>
@@ -2156,28 +2156,28 @@
       <c r="O18" s="7">
         <v>10.24</v>
       </c>
-      <c r="P18" s="30">
+      <c r="P18" s="33">
         <v>6.7</v>
       </c>
-      <c r="Q18" s="28"/>
-      <c r="R18" s="27"/>
+      <c r="Q18" s="34"/>
+      <c r="R18" s="24"/>
       <c r="S18" s="7">
         <v>2.9</v>
       </c>
-      <c r="T18" s="30">
+      <c r="T18" s="33">
         <v>198.96299999999999</v>
       </c>
-      <c r="U18" s="27"/>
+      <c r="U18" s="24"/>
       <c r="V18" s="7">
         <v>68.608000000000004</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A19" s="23"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="25"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
       <c r="F19" s="4" t="s">
         <v>89</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>90</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>14</v>
@@ -2208,28 +2208,28 @@
       <c r="O19" s="7">
         <v>7.3</v>
       </c>
-      <c r="P19" s="30">
+      <c r="P19" s="33">
         <v>7.3</v>
       </c>
-      <c r="Q19" s="28"/>
-      <c r="R19" s="27"/>
+      <c r="Q19" s="34"/>
+      <c r="R19" s="24"/>
       <c r="S19" s="7">
         <v>2.9</v>
       </c>
-      <c r="T19" s="30">
+      <c r="T19" s="33">
         <v>154.541</v>
       </c>
-      <c r="U19" s="27"/>
+      <c r="U19" s="24"/>
       <c r="V19" s="7">
         <v>53.29</v>
       </c>
     </row>
     <row r="20" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="23"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="25"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="22"/>
       <c r="F20" s="4" t="s">
         <v>27</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>91</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>14</v>
@@ -2260,28 +2260,28 @@
       <c r="O20" s="7">
         <v>6.7</v>
       </c>
-      <c r="P20" s="30">
+      <c r="P20" s="33">
         <v>10.25</v>
       </c>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="27"/>
+      <c r="Q20" s="34"/>
+      <c r="R20" s="24"/>
       <c r="S20" s="7">
         <v>2.9</v>
       </c>
-      <c r="T20" s="30">
+      <c r="T20" s="33">
         <v>199.15799999999999</v>
       </c>
-      <c r="U20" s="27"/>
+      <c r="U20" s="24"/>
       <c r="V20" s="7">
         <v>68.674999999999997</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="23"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="25"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4" t="s">
         <v>61</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>92</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>14</v>
@@ -2312,28 +2312,28 @@
       <c r="O21" s="7">
         <v>6.7</v>
       </c>
-      <c r="P21" s="30">
+      <c r="P21" s="33">
         <v>10.95</v>
       </c>
-      <c r="Q21" s="28"/>
-      <c r="R21" s="27"/>
+      <c r="Q21" s="34"/>
+      <c r="R21" s="24"/>
       <c r="S21" s="7">
         <v>2.9</v>
       </c>
-      <c r="T21" s="30">
+      <c r="T21" s="33">
         <v>212.75899999999999</v>
       </c>
-      <c r="U21" s="27"/>
+      <c r="U21" s="24"/>
       <c r="V21" s="7">
         <v>73.364999999999995</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="23"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="25"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="4" t="s">
         <v>28</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>93</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="I22" s="4" t="s">
         <v>14</v>
@@ -2364,30 +2364,30 @@
       <c r="O22" s="7">
         <v>6.7</v>
       </c>
-      <c r="P22" s="30">
+      <c r="P22" s="33">
         <v>11.75</v>
       </c>
-      <c r="Q22" s="28"/>
-      <c r="R22" s="27"/>
+      <c r="Q22" s="34"/>
+      <c r="R22" s="24"/>
       <c r="S22" s="7">
         <v>2.9</v>
       </c>
-      <c r="T22" s="30">
+      <c r="T22" s="33">
         <v>228.303</v>
       </c>
-      <c r="U22" s="27"/>
+      <c r="U22" s="24"/>
       <c r="V22" s="7">
         <v>78.724999999999994</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="23"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="23" t="s">
+      <c r="A23" s="20"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="22"/>
       <c r="F23" s="4" t="s">
         <v>62</v>
       </c>
@@ -2418,28 +2418,28 @@
       <c r="O23" s="7">
         <v>18.649999999999999</v>
       </c>
-      <c r="P23" s="30">
+      <c r="P23" s="33">
         <v>6.65</v>
       </c>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="27"/>
+      <c r="Q23" s="34"/>
+      <c r="R23" s="24"/>
       <c r="S23" s="7">
         <v>3.41</v>
       </c>
-      <c r="T23" s="30">
+      <c r="T23" s="33">
         <v>422.91699999999997</v>
       </c>
-      <c r="U23" s="27"/>
+      <c r="U23" s="24"/>
       <c r="V23" s="7">
         <v>124.023</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="23"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="22"/>
       <c r="F24" s="4" t="s">
         <v>55</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>97</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>14</v>
@@ -2470,28 +2470,28 @@
       <c r="O24" s="7">
         <v>7.47</v>
       </c>
-      <c r="P24" s="30">
+      <c r="P24" s="33">
         <v>6.68</v>
       </c>
-      <c r="Q24" s="28"/>
-      <c r="R24" s="27"/>
+      <c r="Q24" s="34"/>
+      <c r="R24" s="24"/>
       <c r="S24" s="7">
         <v>3.39</v>
       </c>
-      <c r="T24" s="30">
+      <c r="T24" s="33">
         <v>169.16</v>
       </c>
-      <c r="U24" s="27"/>
+      <c r="U24" s="24"/>
       <c r="V24" s="7">
         <v>49.9</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="23"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="25"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
       <c r="F25" s="4" t="s">
         <v>98</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>99</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>181</v>
+        <v>156</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>14</v>
@@ -2522,28 +2522,28 @@
       <c r="O25" s="7">
         <v>7.38</v>
       </c>
-      <c r="P25" s="30">
+      <c r="P25" s="33">
         <v>6.68</v>
       </c>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="27"/>
+      <c r="Q25" s="34"/>
+      <c r="R25" s="24"/>
       <c r="S25" s="7">
         <v>3.43</v>
       </c>
-      <c r="T25" s="30">
+      <c r="T25" s="33">
         <v>169.09399999999999</v>
       </c>
-      <c r="U25" s="27"/>
+      <c r="U25" s="24"/>
       <c r="V25" s="7">
         <v>49.298000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="23"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="25"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="22"/>
       <c r="F26" s="4" t="s">
         <v>100</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>101</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>14</v>
@@ -2574,28 +2574,28 @@
       <c r="O26" s="7">
         <v>14.92</v>
       </c>
-      <c r="P26" s="30">
+      <c r="P26" s="33">
         <v>6.68</v>
       </c>
-      <c r="Q26" s="28"/>
-      <c r="R26" s="27"/>
+      <c r="Q26" s="34"/>
+      <c r="R26" s="24"/>
       <c r="S26" s="7">
         <v>3.43</v>
       </c>
-      <c r="T26" s="30">
+      <c r="T26" s="33">
         <v>341.85300000000001</v>
       </c>
-      <c r="U26" s="27"/>
+      <c r="U26" s="24"/>
       <c r="V26" s="7">
         <v>99.665999999999997</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="23"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="25"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="22"/>
       <c r="F27" s="4" t="s">
         <v>18</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>102</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>14</v>
@@ -2626,28 +2626,28 @@
       <c r="O27" s="7">
         <v>10.97</v>
       </c>
-      <c r="P27" s="30">
+      <c r="P27" s="33">
         <v>6.64</v>
       </c>
-      <c r="Q27" s="28"/>
-      <c r="R27" s="27"/>
+      <c r="Q27" s="34"/>
+      <c r="R27" s="24"/>
       <c r="S27" s="7">
         <v>3.31</v>
       </c>
-      <c r="T27" s="30">
+      <c r="T27" s="33">
         <v>241.10300000000001</v>
       </c>
-      <c r="U27" s="27"/>
+      <c r="U27" s="24"/>
       <c r="V27" s="7">
         <v>72.840999999999994</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A28" s="23"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="25"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="22"/>
       <c r="F28" s="4" t="s">
         <v>64</v>
       </c>
@@ -2655,10 +2655,10 @@
         <v>103</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>29</v>
@@ -2678,28 +2678,28 @@
       <c r="O28" s="7">
         <v>18.98</v>
       </c>
-      <c r="P28" s="30">
+      <c r="P28" s="33">
         <v>6.64</v>
       </c>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="27"/>
+      <c r="Q28" s="34"/>
+      <c r="R28" s="24"/>
       <c r="S28" s="7">
         <v>3.31</v>
       </c>
-      <c r="T28" s="30">
+      <c r="T28" s="33">
         <v>417.15</v>
       </c>
-      <c r="U28" s="27"/>
+      <c r="U28" s="24"/>
       <c r="V28" s="7">
         <v>126.027</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="23"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="25"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="22"/>
       <c r="F29" s="4" t="s">
         <v>21</v>
       </c>
@@ -2728,28 +2728,28 @@
       <c r="O29" s="7">
         <v>11.03</v>
       </c>
-      <c r="P29" s="30">
+      <c r="P29" s="33">
         <v>6.79</v>
       </c>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="27"/>
+      <c r="Q29" s="34"/>
+      <c r="R29" s="24"/>
       <c r="S29" s="7">
         <v>3.14</v>
       </c>
-      <c r="T29" s="30">
+      <c r="T29" s="33">
         <v>235.166</v>
       </c>
-      <c r="U29" s="27"/>
+      <c r="U29" s="24"/>
       <c r="V29" s="7">
         <v>74.894000000000005</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="23"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="25"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="22"/>
       <c r="F30" s="4" t="s">
         <v>23</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>105</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I30" s="4" t="s">
         <v>14</v>
@@ -2780,30 +2780,30 @@
       <c r="O30" s="7">
         <v>6.77</v>
       </c>
-      <c r="P30" s="30">
+      <c r="P30" s="33">
         <v>11.02</v>
       </c>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="27"/>
+      <c r="Q30" s="34"/>
+      <c r="R30" s="24"/>
       <c r="S30" s="7">
         <v>2.95</v>
       </c>
-      <c r="T30" s="30">
+      <c r="T30" s="33">
         <v>220.08600000000001</v>
       </c>
-      <c r="U30" s="27"/>
+      <c r="U30" s="24"/>
       <c r="V30" s="7">
         <v>74.605000000000004</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A31" s="23"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="23" t="s">
+      <c r="A31" s="20"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="25"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="22"/>
       <c r="F31" s="4" t="s">
         <v>64</v>
       </c>
@@ -2832,28 +2832,28 @@
       <c r="O31" s="7">
         <v>22.46</v>
       </c>
-      <c r="P31" s="30">
+      <c r="P31" s="33">
         <v>6.68</v>
       </c>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="27"/>
+      <c r="Q31" s="34"/>
+      <c r="R31" s="24"/>
       <c r="S31" s="7">
         <v>3.25</v>
       </c>
-      <c r="T31" s="30">
+      <c r="T31" s="33">
         <v>487.60700000000003</v>
       </c>
-      <c r="U31" s="27"/>
+      <c r="U31" s="24"/>
       <c r="V31" s="7">
         <v>150.03299999999999</v>
       </c>
     </row>
     <row r="32" spans="1:22" ht="52.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="23"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="25"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="22"/>
       <c r="F32" s="4" t="s">
         <v>44</v>
       </c>
@@ -2882,28 +2882,28 @@
       <c r="O32" s="7">
         <v>18.75</v>
       </c>
-      <c r="P32" s="30">
+      <c r="P32" s="33">
         <v>6.46</v>
       </c>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="27"/>
+      <c r="Q32" s="34"/>
+      <c r="R32" s="24"/>
       <c r="S32" s="7">
         <v>3.26</v>
       </c>
-      <c r="T32" s="30">
+      <c r="T32" s="33">
         <v>394.86799999999999</v>
       </c>
-      <c r="U32" s="27"/>
+      <c r="U32" s="24"/>
       <c r="V32" s="7">
         <v>121.125</v>
       </c>
     </row>
     <row r="33" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="23"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="25"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="22"/>
       <c r="F33" s="4" t="s">
         <v>16</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>109</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="I33" s="4" t="s">
         <v>14</v>
@@ -2934,28 +2934,28 @@
       <c r="O33" s="7">
         <v>13.55</v>
       </c>
-      <c r="P33" s="30">
+      <c r="P33" s="33">
         <v>6.8</v>
       </c>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="27"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="24"/>
       <c r="S33" s="7">
         <v>2.95</v>
       </c>
-      <c r="T33" s="30">
+      <c r="T33" s="33">
         <v>271.81299999999999</v>
       </c>
-      <c r="U33" s="27"/>
+      <c r="U33" s="24"/>
       <c r="V33" s="7">
         <v>92.14</v>
       </c>
     </row>
     <row r="34" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A34" s="23"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="25"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="22"/>
       <c r="F34" s="4" t="s">
         <v>110</v>
       </c>
@@ -2963,10 +2963,10 @@
         <v>111</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>29</v>
@@ -2986,28 +2986,28 @@
       <c r="O34" s="7">
         <v>13.3</v>
       </c>
-      <c r="P34" s="30">
+      <c r="P34" s="33">
         <v>6.8</v>
       </c>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="27"/>
+      <c r="Q34" s="34"/>
+      <c r="R34" s="24"/>
       <c r="S34" s="7">
         <v>2.95</v>
       </c>
-      <c r="T34" s="30">
+      <c r="T34" s="33">
         <v>266.798</v>
       </c>
-      <c r="U34" s="27"/>
+      <c r="U34" s="24"/>
       <c r="V34" s="7">
         <v>90.44</v>
       </c>
     </row>
     <row r="35" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A35" s="23"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="25"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="22"/>
       <c r="F35" s="4" t="s">
         <v>54</v>
       </c>
@@ -3036,28 +3036,28 @@
       <c r="O35" s="7">
         <v>2.59</v>
       </c>
-      <c r="P35" s="30">
+      <c r="P35" s="33">
         <v>6.78</v>
       </c>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="27"/>
+      <c r="Q35" s="34"/>
+      <c r="R35" s="24"/>
       <c r="S35" s="7">
         <v>2.94</v>
       </c>
-      <c r="T35" s="30">
+      <c r="T35" s="33">
         <v>51.627000000000002</v>
       </c>
-      <c r="U35" s="27"/>
+      <c r="U35" s="24"/>
       <c r="V35" s="7">
         <v>17.559999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A36" s="23"/>
-      <c r="B36" s="25"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="25"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="22"/>
       <c r="F36" s="4" t="s">
         <v>56</v>
       </c>
@@ -3086,28 +3086,28 @@
       <c r="O36" s="7">
         <v>22.35</v>
       </c>
-      <c r="P36" s="30">
+      <c r="P36" s="33">
         <v>6.85</v>
       </c>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="27"/>
+      <c r="Q36" s="34"/>
+      <c r="R36" s="24"/>
       <c r="S36" s="7">
         <v>2.94</v>
       </c>
-      <c r="T36" s="30">
+      <c r="T36" s="33">
         <v>450.10700000000003</v>
       </c>
-      <c r="U36" s="27"/>
+      <c r="U36" s="24"/>
       <c r="V36" s="7">
         <v>153.09800000000001</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A37" s="23"/>
-      <c r="B37" s="25"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="25"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="22"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="22"/>
       <c r="F37" s="4" t="s">
         <v>73</v>
       </c>
@@ -3115,10 +3115,10 @@
         <v>114</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="J37" s="4" t="s">
         <v>29</v>
@@ -3138,28 +3138,28 @@
       <c r="O37" s="7">
         <v>13.55</v>
       </c>
-      <c r="P37" s="30">
+      <c r="P37" s="33">
         <v>6.8</v>
       </c>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="27"/>
+      <c r="Q37" s="34"/>
+      <c r="R37" s="24"/>
       <c r="S37" s="7">
         <v>2.95</v>
       </c>
-      <c r="T37" s="30">
+      <c r="T37" s="33">
         <v>271.81299999999999</v>
       </c>
-      <c r="U37" s="27"/>
+      <c r="U37" s="24"/>
       <c r="V37" s="7">
         <v>92.14</v>
       </c>
     </row>
     <row r="38" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="23"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="25"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="22"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="22"/>
       <c r="F38" s="4" t="s">
         <v>24</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>115</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>116</v>
+        <v>181</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>14</v>
@@ -3190,36 +3190,36 @@
       <c r="O38" s="7">
         <v>13.22</v>
       </c>
-      <c r="P38" s="30">
+      <c r="P38" s="33">
         <v>6.8</v>
       </c>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="27"/>
+      <c r="Q38" s="34"/>
+      <c r="R38" s="24"/>
       <c r="S38" s="7">
         <v>2.94</v>
       </c>
-      <c r="T38" s="30">
+      <c r="T38" s="33">
         <v>264.29399999999998</v>
       </c>
-      <c r="U38" s="27"/>
+      <c r="U38" s="24"/>
       <c r="V38" s="7">
         <v>89.896000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A39" s="23"/>
-      <c r="B39" s="25"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="25"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="22"/>
       <c r="F39" s="4" t="s">
         <v>49</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>118</v>
+        <v>182</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>14</v>
@@ -3242,36 +3242,36 @@
       <c r="O39" s="7">
         <v>11.23</v>
       </c>
-      <c r="P39" s="30">
+      <c r="P39" s="33">
         <v>6.8</v>
       </c>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="27"/>
+      <c r="Q39" s="34"/>
+      <c r="R39" s="24"/>
       <c r="S39" s="7">
         <v>2.94</v>
       </c>
-      <c r="T39" s="30">
+      <c r="T39" s="33">
         <v>224.51</v>
       </c>
-      <c r="U39" s="27"/>
+      <c r="U39" s="24"/>
       <c r="V39" s="7">
         <v>76.364000000000004</v>
       </c>
     </row>
     <row r="40" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="23"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="25"/>
+      <c r="A40" s="20"/>
+      <c r="B40" s="22"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="22"/>
       <c r="F40" s="4" t="s">
         <v>50</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>14</v>
@@ -3294,36 +3294,36 @@
       <c r="O40" s="7">
         <v>11.19</v>
       </c>
-      <c r="P40" s="30">
+      <c r="P40" s="33">
         <v>6.79</v>
       </c>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="27"/>
+      <c r="Q40" s="34"/>
+      <c r="R40" s="24"/>
       <c r="S40" s="7">
         <v>2.92</v>
       </c>
-      <c r="T40" s="30">
+      <c r="T40" s="33">
         <v>221.86199999999999</v>
       </c>
-      <c r="U40" s="27"/>
+      <c r="U40" s="24"/>
       <c r="V40" s="7">
         <v>75.98</v>
       </c>
     </row>
     <row r="41" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="23"/>
-      <c r="B41" s="25"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="25"/>
+      <c r="A41" s="20"/>
+      <c r="B41" s="22"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="22"/>
       <c r="F41" s="4" t="s">
         <v>59</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>122</v>
+        <v>184</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>14</v>
@@ -3346,36 +3346,36 @@
       <c r="O41" s="7">
         <v>11.13</v>
       </c>
-      <c r="P41" s="30">
+      <c r="P41" s="33">
         <v>6.81</v>
       </c>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="27"/>
+      <c r="Q41" s="34"/>
+      <c r="R41" s="24"/>
       <c r="S41" s="7">
         <v>2.96</v>
       </c>
-      <c r="T41" s="30">
+      <c r="T41" s="33">
         <v>224.35400000000001</v>
       </c>
-      <c r="U41" s="27"/>
+      <c r="U41" s="24"/>
       <c r="V41" s="7">
         <v>75.795000000000002</v>
       </c>
     </row>
     <row r="42" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="23"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="25"/>
+      <c r="A42" s="20"/>
+      <c r="B42" s="22"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="22"/>
       <c r="F42" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>124</v>
+        <v>185</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>14</v>
@@ -3398,36 +3398,36 @@
       <c r="O42" s="7">
         <v>10.94</v>
       </c>
-      <c r="P42" s="30">
+      <c r="P42" s="33">
         <v>6.91</v>
       </c>
-      <c r="Q42" s="28"/>
-      <c r="R42" s="27"/>
+      <c r="Q42" s="34"/>
+      <c r="R42" s="24"/>
       <c r="S42" s="7">
         <v>2.96</v>
       </c>
-      <c r="T42" s="30">
+      <c r="T42" s="33">
         <v>223.762</v>
       </c>
-      <c r="U42" s="27"/>
+      <c r="U42" s="24"/>
       <c r="V42" s="7">
         <v>75.594999999999999</v>
       </c>
     </row>
     <row r="43" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="23"/>
-      <c r="B43" s="25"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="25"/>
+      <c r="A43" s="20"/>
+      <c r="B43" s="22"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="22"/>
       <c r="F43" s="4" t="s">
         <v>52</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>14</v>
@@ -3450,33 +3450,33 @@
       <c r="O43" s="7">
         <v>13.62</v>
       </c>
-      <c r="P43" s="30">
+      <c r="P43" s="33">
         <v>6.81</v>
       </c>
-      <c r="Q43" s="28"/>
-      <c r="R43" s="27"/>
+      <c r="Q43" s="34"/>
+      <c r="R43" s="24"/>
       <c r="S43" s="7">
         <v>2.96</v>
       </c>
-      <c r="T43" s="30">
+      <c r="T43" s="33">
         <v>274.54700000000003</v>
       </c>
-      <c r="U43" s="27"/>
+      <c r="U43" s="24"/>
       <c r="V43" s="7">
         <v>92.751999999999995</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="23"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="25"/>
+      <c r="A44" s="20"/>
+      <c r="B44" s="22"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="22"/>
       <c r="F44" s="4" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="4" t="s">
@@ -3500,35 +3500,35 @@
       <c r="O44" s="7">
         <v>7.47</v>
       </c>
-      <c r="P44" s="30">
+      <c r="P44" s="33">
         <v>7.37</v>
       </c>
-      <c r="Q44" s="28"/>
-      <c r="R44" s="27"/>
+      <c r="Q44" s="34"/>
+      <c r="R44" s="24"/>
       <c r="S44" s="7">
         <v>2.64</v>
       </c>
-      <c r="T44" s="30">
+      <c r="T44" s="33">
         <v>145.34200000000001</v>
       </c>
-      <c r="U44" s="27"/>
+      <c r="U44" s="24"/>
       <c r="V44" s="7">
         <v>55.054000000000002</v>
       </c>
     </row>
     <row r="45" spans="1:22" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="23"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="D45" s="24"/>
-      <c r="E45" s="25"/>
+      <c r="A45" s="20"/>
+      <c r="B45" s="22"/>
+      <c r="C45" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D45" s="21"/>
+      <c r="E45" s="22"/>
       <c r="F45" s="4" t="s">
         <v>98</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="4" t="s">
@@ -3552,33 +3552,33 @@
       <c r="O45" s="7">
         <v>4.87</v>
       </c>
-      <c r="P45" s="30">
+      <c r="P45" s="33">
         <v>7.53</v>
       </c>
-      <c r="Q45" s="28"/>
-      <c r="R45" s="27"/>
+      <c r="Q45" s="34"/>
+      <c r="R45" s="24"/>
       <c r="S45" s="7">
         <v>2.92</v>
       </c>
-      <c r="T45" s="30">
+      <c r="T45" s="33">
         <v>107.08</v>
       </c>
-      <c r="U45" s="27"/>
+      <c r="U45" s="24"/>
       <c r="V45" s="7">
         <v>36.670999999999999</v>
       </c>
     </row>
     <row r="46" spans="1:22" ht="21" x14ac:dyDescent="0.35">
-      <c r="A46" s="23"/>
-      <c r="B46" s="25"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="25"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="22"/>
       <c r="F46" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="4" t="s">
@@ -3602,33 +3602,33 @@
       <c r="O46" s="7">
         <v>11.33</v>
       </c>
-      <c r="P46" s="30">
+      <c r="P46" s="33">
         <v>8.77</v>
       </c>
-      <c r="Q46" s="28"/>
-      <c r="R46" s="27"/>
+      <c r="Q46" s="34"/>
+      <c r="R46" s="24"/>
       <c r="S46" s="7">
         <v>3.07</v>
       </c>
-      <c r="T46" s="30">
+      <c r="T46" s="33">
         <v>305.048</v>
       </c>
-      <c r="U46" s="27"/>
+      <c r="U46" s="24"/>
       <c r="V46" s="7">
         <v>99.364000000000004</v>
       </c>
     </row>
     <row r="47" spans="1:22" ht="21" x14ac:dyDescent="0.35">
-      <c r="A47" s="23"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="25"/>
+      <c r="A47" s="20"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="22"/>
       <c r="F47" s="4" t="s">
         <v>37</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
@@ -3652,33 +3652,33 @@
       <c r="O47" s="7">
         <v>7.9</v>
       </c>
-      <c r="P47" s="30">
+      <c r="P47" s="33">
         <v>8.85</v>
       </c>
-      <c r="Q47" s="28"/>
-      <c r="R47" s="27"/>
+      <c r="Q47" s="34"/>
+      <c r="R47" s="24"/>
       <c r="S47" s="7">
         <v>3.07</v>
       </c>
-      <c r="T47" s="30">
+      <c r="T47" s="33">
         <v>214.63900000000001</v>
       </c>
-      <c r="U47" s="27"/>
+      <c r="U47" s="24"/>
       <c r="V47" s="7">
         <v>69.915000000000006</v>
       </c>
     </row>
     <row r="48" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="23"/>
-      <c r="B48" s="25"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="25"/>
+      <c r="A48" s="20"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="22"/>
       <c r="F48" s="4" t="s">
         <v>63</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
@@ -3702,33 +3702,33 @@
       <c r="O48" s="7">
         <v>8</v>
       </c>
-      <c r="P48" s="30">
+      <c r="P48" s="33">
         <v>8.85</v>
       </c>
-      <c r="Q48" s="28"/>
-      <c r="R48" s="27"/>
+      <c r="Q48" s="34"/>
+      <c r="R48" s="24"/>
       <c r="S48" s="7">
         <v>3.07</v>
       </c>
-      <c r="T48" s="30">
+      <c r="T48" s="33">
         <v>217.35599999999999</v>
       </c>
-      <c r="U48" s="27"/>
+      <c r="U48" s="24"/>
       <c r="V48" s="7">
         <v>70.8</v>
       </c>
     </row>
     <row r="49" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="23"/>
-      <c r="B49" s="25"/>
-      <c r="C49" s="23"/>
-      <c r="D49" s="24"/>
-      <c r="E49" s="25"/>
+      <c r="A49" s="20"/>
+      <c r="B49" s="22"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="22"/>
       <c r="F49" s="4" t="s">
         <v>60</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="4" t="s">
@@ -3752,33 +3752,33 @@
       <c r="O49" s="7">
         <v>7.52</v>
       </c>
-      <c r="P49" s="30">
+      <c r="P49" s="33">
         <v>10.73</v>
       </c>
-      <c r="Q49" s="28"/>
-      <c r="R49" s="27"/>
+      <c r="Q49" s="34"/>
+      <c r="R49" s="24"/>
       <c r="S49" s="7">
         <v>3.16</v>
       </c>
-      <c r="T49" s="30">
+      <c r="T49" s="33">
         <v>254.97900000000001</v>
       </c>
-      <c r="U49" s="27"/>
+      <c r="U49" s="24"/>
       <c r="V49" s="7">
         <v>80.69</v>
       </c>
     </row>
     <row r="50" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="23"/>
-      <c r="B50" s="25"/>
-      <c r="C50" s="23"/>
-      <c r="D50" s="24"/>
-      <c r="E50" s="25"/>
+      <c r="A50" s="20"/>
+      <c r="B50" s="22"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="21"/>
+      <c r="E50" s="22"/>
       <c r="F50" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4" t="s">
@@ -3802,33 +3802,33 @@
       <c r="O50" s="7">
         <v>7.54</v>
       </c>
-      <c r="P50" s="30">
+      <c r="P50" s="33">
         <v>10.66</v>
       </c>
-      <c r="Q50" s="28"/>
-      <c r="R50" s="27"/>
+      <c r="Q50" s="34"/>
+      <c r="R50" s="24"/>
       <c r="S50" s="7">
         <v>3.16</v>
       </c>
-      <c r="T50" s="30">
+      <c r="T50" s="33">
         <v>253.989</v>
       </c>
-      <c r="U50" s="27"/>
+      <c r="U50" s="24"/>
       <c r="V50" s="7">
         <v>80.376000000000005</v>
       </c>
     </row>
     <row r="51" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="23"/>
-      <c r="B51" s="25"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="25"/>
+      <c r="A51" s="20"/>
+      <c r="B51" s="22"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="22"/>
       <c r="F51" s="4" t="s">
         <v>45</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
@@ -3852,33 +3852,33 @@
       <c r="O51" s="7">
         <v>7.59</v>
       </c>
-      <c r="P51" s="30">
+      <c r="P51" s="33">
         <v>11.48</v>
       </c>
-      <c r="Q51" s="28"/>
-      <c r="R51" s="27"/>
+      <c r="Q51" s="34"/>
+      <c r="R51" s="24"/>
       <c r="S51" s="7">
         <v>3.07</v>
       </c>
-      <c r="T51" s="30">
+      <c r="T51" s="33">
         <v>267.49900000000002</v>
       </c>
-      <c r="U51" s="27"/>
+      <c r="U51" s="24"/>
       <c r="V51" s="7">
         <v>87.132999999999996</v>
       </c>
     </row>
     <row r="52" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="23"/>
-      <c r="B52" s="25"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="24"/>
-      <c r="E52" s="25"/>
+      <c r="A52" s="20"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="22"/>
       <c r="F52" s="4" t="s">
         <v>46</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
@@ -3902,33 +3902,33 @@
       <c r="O52" s="7">
         <v>7.57</v>
       </c>
-      <c r="P52" s="30">
+      <c r="P52" s="33">
         <v>7.74</v>
       </c>
-      <c r="Q52" s="28"/>
-      <c r="R52" s="27"/>
+      <c r="Q52" s="34"/>
+      <c r="R52" s="24"/>
       <c r="S52" s="7">
         <v>3.07</v>
       </c>
-      <c r="T52" s="30">
+      <c r="T52" s="33">
         <v>179.87700000000001</v>
       </c>
-      <c r="U52" s="27"/>
+      <c r="U52" s="24"/>
       <c r="V52" s="7">
         <v>58.591999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="23"/>
-      <c r="B53" s="25"/>
-      <c r="C53" s="23"/>
-      <c r="D53" s="24"/>
-      <c r="E53" s="25"/>
+      <c r="A53" s="20"/>
+      <c r="B53" s="22"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="22"/>
       <c r="F53" s="4" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
@@ -3952,33 +3952,33 @@
       <c r="O53" s="7">
         <v>4.5</v>
       </c>
-      <c r="P53" s="30">
+      <c r="P53" s="33">
         <v>7.77</v>
       </c>
-      <c r="Q53" s="28"/>
-      <c r="R53" s="27"/>
+      <c r="Q53" s="34"/>
+      <c r="R53" s="24"/>
       <c r="S53" s="7">
         <v>3.21</v>
       </c>
-      <c r="T53" s="30">
+      <c r="T53" s="33">
         <v>112.238</v>
       </c>
-      <c r="U53" s="27"/>
+      <c r="U53" s="24"/>
       <c r="V53" s="7">
         <v>34.965000000000003</v>
       </c>
     </row>
     <row r="54" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="23"/>
-      <c r="B54" s="25"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="24"/>
-      <c r="E54" s="25"/>
+      <c r="A54" s="20"/>
+      <c r="B54" s="22"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="21"/>
+      <c r="E54" s="22"/>
       <c r="F54" s="4" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
@@ -4002,33 +4002,33 @@
       <c r="O54" s="7">
         <v>7.08</v>
       </c>
-      <c r="P54" s="30">
+      <c r="P54" s="33">
         <v>7</v>
       </c>
-      <c r="Q54" s="28"/>
-      <c r="R54" s="27"/>
+      <c r="Q54" s="34"/>
+      <c r="R54" s="24"/>
       <c r="S54" s="7">
         <v>3.2</v>
       </c>
-      <c r="T54" s="30">
+      <c r="T54" s="33">
         <v>158.59200000000001</v>
       </c>
-      <c r="U54" s="27"/>
+      <c r="U54" s="24"/>
       <c r="V54" s="7">
         <v>49.56</v>
       </c>
     </row>
     <row r="55" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="23"/>
-      <c r="B55" s="25"/>
-      <c r="C55" s="23"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="25"/>
+      <c r="A55" s="20"/>
+      <c r="B55" s="22"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="22"/>
       <c r="F55" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
@@ -4052,33 +4052,33 @@
       <c r="O55" s="7">
         <v>7</v>
       </c>
-      <c r="P55" s="30">
+      <c r="P55" s="33">
         <v>7.8</v>
       </c>
-      <c r="Q55" s="28"/>
-      <c r="R55" s="27"/>
+      <c r="Q55" s="34"/>
+      <c r="R55" s="24"/>
       <c r="S55" s="7">
         <v>3.22</v>
       </c>
-      <c r="T55" s="30">
+      <c r="T55" s="33">
         <v>175.81200000000001</v>
       </c>
-      <c r="U55" s="27"/>
+      <c r="U55" s="24"/>
       <c r="V55" s="7">
         <v>54.6</v>
       </c>
     </row>
     <row r="56" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="23"/>
-      <c r="B56" s="25"/>
-      <c r="C56" s="23"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="25"/>
+      <c r="A56" s="20"/>
+      <c r="B56" s="22"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="21"/>
+      <c r="E56" s="22"/>
       <c r="F56" s="4" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
@@ -4102,33 +4102,33 @@
       <c r="O56" s="7">
         <v>7</v>
       </c>
-      <c r="P56" s="30">
+      <c r="P56" s="33">
         <v>8</v>
       </c>
-      <c r="Q56" s="28"/>
-      <c r="R56" s="27"/>
+      <c r="Q56" s="34"/>
+      <c r="R56" s="24"/>
       <c r="S56" s="7">
         <v>3.22</v>
       </c>
-      <c r="T56" s="30">
+      <c r="T56" s="33">
         <v>180.32</v>
       </c>
-      <c r="U56" s="27"/>
+      <c r="U56" s="24"/>
       <c r="V56" s="7">
         <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A57" s="23"/>
-      <c r="B57" s="25"/>
-      <c r="C57" s="23"/>
-      <c r="D57" s="24"/>
-      <c r="E57" s="25"/>
+      <c r="A57" s="20"/>
+      <c r="B57" s="22"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="21"/>
+      <c r="E57" s="22"/>
       <c r="F57" s="4" t="s">
         <v>47</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
@@ -4152,33 +4152,33 @@
       <c r="O57" s="7">
         <v>7.75</v>
       </c>
-      <c r="P57" s="30">
+      <c r="P57" s="33">
         <v>8.7799999999999994</v>
       </c>
-      <c r="Q57" s="28"/>
-      <c r="R57" s="27"/>
+      <c r="Q57" s="34"/>
+      <c r="R57" s="24"/>
       <c r="S57" s="7">
         <v>2.97</v>
       </c>
-      <c r="T57" s="30">
+      <c r="T57" s="33">
         <v>202.09399999999999</v>
       </c>
-      <c r="U57" s="27"/>
+      <c r="U57" s="24"/>
       <c r="V57" s="7">
         <v>68.045000000000002</v>
       </c>
     </row>
     <row r="58" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A58" s="23"/>
-      <c r="B58" s="25"/>
-      <c r="C58" s="23"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="25"/>
+      <c r="A58" s="20"/>
+      <c r="B58" s="22"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="21"/>
+      <c r="E58" s="22"/>
       <c r="F58" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
@@ -4202,33 +4202,33 @@
       <c r="O58" s="7">
         <v>5.54</v>
       </c>
-      <c r="P58" s="30">
+      <c r="P58" s="33">
         <v>8.81</v>
       </c>
-      <c r="Q58" s="28"/>
-      <c r="R58" s="27"/>
+      <c r="Q58" s="34"/>
+      <c r="R58" s="24"/>
       <c r="S58" s="7">
         <v>2.94</v>
       </c>
-      <c r="T58" s="30">
+      <c r="T58" s="33">
         <v>143.494</v>
       </c>
-      <c r="U58" s="27"/>
+      <c r="U58" s="24"/>
       <c r="V58" s="7">
         <v>48.807000000000002</v>
       </c>
     </row>
     <row r="59" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A59" s="23"/>
-      <c r="B59" s="25"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="24"/>
-      <c r="E59" s="25"/>
+      <c r="A59" s="20"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="21"/>
+      <c r="E59" s="22"/>
       <c r="F59" s="4" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
@@ -4252,33 +4252,33 @@
       <c r="O59" s="7">
         <v>7.5</v>
       </c>
-      <c r="P59" s="30">
+      <c r="P59" s="33">
         <v>10.77</v>
       </c>
-      <c r="Q59" s="28"/>
-      <c r="R59" s="27"/>
+      <c r="Q59" s="34"/>
+      <c r="R59" s="24"/>
       <c r="S59" s="7">
         <v>2.95</v>
       </c>
-      <c r="T59" s="30">
+      <c r="T59" s="33">
         <v>238.286</v>
       </c>
-      <c r="U59" s="27"/>
+      <c r="U59" s="24"/>
       <c r="V59" s="7">
         <v>80.775000000000006</v>
       </c>
     </row>
     <row r="60" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A60" s="23"/>
-      <c r="B60" s="25"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="24"/>
-      <c r="E60" s="25"/>
+      <c r="A60" s="20"/>
+      <c r="B60" s="22"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="21"/>
+      <c r="E60" s="22"/>
       <c r="F60" s="4" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H60" s="4"/>
       <c r="I60" s="4" t="s">
@@ -4302,33 +4302,33 @@
       <c r="O60" s="7">
         <v>7.6</v>
       </c>
-      <c r="P60" s="30">
+      <c r="P60" s="33">
         <v>8</v>
       </c>
-      <c r="Q60" s="28"/>
-      <c r="R60" s="27"/>
+      <c r="Q60" s="34"/>
+      <c r="R60" s="24"/>
       <c r="S60" s="7">
         <v>3.11</v>
       </c>
-      <c r="T60" s="30">
+      <c r="T60" s="33">
         <v>189.08799999999999</v>
       </c>
-      <c r="U60" s="27"/>
+      <c r="U60" s="24"/>
       <c r="V60" s="7">
         <v>60.8</v>
       </c>
     </row>
     <row r="61" spans="1:22" ht="42" x14ac:dyDescent="0.35">
-      <c r="A61" s="23"/>
-      <c r="B61" s="25"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="24"/>
-      <c r="E61" s="25"/>
+      <c r="A61" s="20"/>
+      <c r="B61" s="22"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="21"/>
+      <c r="E61" s="22"/>
       <c r="F61" s="4" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="H61" s="4"/>
       <c r="I61" s="4" t="s">
@@ -4352,33 +4352,33 @@
       <c r="O61" s="7">
         <v>7.6</v>
       </c>
-      <c r="P61" s="30">
+      <c r="P61" s="33">
         <v>7.78</v>
       </c>
-      <c r="Q61" s="28"/>
-      <c r="R61" s="27"/>
+      <c r="Q61" s="34"/>
+      <c r="R61" s="24"/>
       <c r="S61" s="7">
         <v>3.27</v>
       </c>
-      <c r="T61" s="30">
+      <c r="T61" s="33">
         <v>193.34899999999999</v>
       </c>
-      <c r="U61" s="27"/>
+      <c r="U61" s="24"/>
       <c r="V61" s="7">
         <v>59.128</v>
       </c>
     </row>
     <row r="62" spans="1:22" ht="21" x14ac:dyDescent="0.35">
-      <c r="A62" s="23"/>
-      <c r="B62" s="25"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="24"/>
-      <c r="E62" s="25"/>
+      <c r="A62" s="20"/>
+      <c r="B62" s="22"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="21"/>
+      <c r="E62" s="22"/>
       <c r="F62" s="4" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="H62" s="4"/>
       <c r="I62" s="4" t="s">
@@ -4402,33 +4402,33 @@
       <c r="O62" s="7">
         <v>6.18</v>
       </c>
-      <c r="P62" s="30">
+      <c r="P62" s="33">
         <v>7.54</v>
       </c>
-      <c r="Q62" s="28"/>
-      <c r="R62" s="27"/>
+      <c r="Q62" s="34"/>
+      <c r="R62" s="24"/>
       <c r="S62" s="7">
         <v>3.12</v>
       </c>
-      <c r="T62" s="30">
+      <c r="T62" s="33">
         <v>145.38300000000001</v>
       </c>
-      <c r="U62" s="27"/>
+      <c r="U62" s="24"/>
       <c r="V62" s="7">
         <v>46.597000000000001</v>
       </c>
     </row>
     <row r="63" spans="1:22" ht="21" x14ac:dyDescent="0.35">
-      <c r="A63" s="23"/>
-      <c r="B63" s="25"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="25"/>
+      <c r="A63" s="20"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="21"/>
+      <c r="E63" s="22"/>
       <c r="F63" s="4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="4" t="s">
@@ -4452,417 +4452,417 @@
       <c r="O63" s="7">
         <v>4.63</v>
       </c>
-      <c r="P63" s="30">
+      <c r="P63" s="33">
         <v>7.85</v>
       </c>
-      <c r="Q63" s="28"/>
-      <c r="R63" s="27"/>
+      <c r="Q63" s="34"/>
+      <c r="R63" s="24"/>
       <c r="S63" s="7">
         <v>3.22</v>
       </c>
-      <c r="T63" s="30">
+      <c r="T63" s="33">
         <v>117.033</v>
       </c>
-      <c r="U63" s="27"/>
+      <c r="U63" s="24"/>
       <c r="V63" s="7">
         <v>36.345999999999997</v>
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A64" s="23"/>
-      <c r="B64" s="25"/>
+      <c r="A64" s="20"/>
+      <c r="B64" s="22"/>
       <c r="C64" s="13"/>
       <c r="D64" s="15"/>
       <c r="E64" s="14"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A65" s="23"/>
-      <c r="B65" s="25"/>
+      <c r="A65" s="20"/>
+      <c r="B65" s="22"/>
       <c r="C65" s="13"/>
       <c r="D65" s="15"/>
       <c r="E65" s="14"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66" s="23"/>
-      <c r="B66" s="25"/>
+      <c r="A66" s="20"/>
+      <c r="B66" s="22"/>
       <c r="C66" s="13"/>
       <c r="D66" s="15"/>
       <c r="E66" s="14"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A67" s="23"/>
-      <c r="B67" s="25"/>
+      <c r="A67" s="20"/>
+      <c r="B67" s="22"/>
       <c r="C67" s="13"/>
       <c r="D67" s="15"/>
       <c r="E67" s="14"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A68" s="23"/>
-      <c r="B68" s="25"/>
+      <c r="A68" s="20"/>
+      <c r="B68" s="22"/>
       <c r="C68" s="13"/>
       <c r="D68" s="15"/>
       <c r="E68" s="14"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A69" s="23"/>
-      <c r="B69" s="25"/>
+      <c r="A69" s="20"/>
+      <c r="B69" s="22"/>
       <c r="C69" s="13"/>
       <c r="D69" s="15"/>
       <c r="E69" s="14"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A70" s="23"/>
-      <c r="B70" s="25"/>
+      <c r="A70" s="20"/>
+      <c r="B70" s="22"/>
       <c r="C70" s="13"/>
       <c r="D70" s="15"/>
       <c r="E70" s="14"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A71" s="23"/>
-      <c r="B71" s="25"/>
+      <c r="A71" s="20"/>
+      <c r="B71" s="22"/>
       <c r="C71" s="13"/>
       <c r="D71" s="15"/>
       <c r="E71" s="14"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A72" s="23"/>
-      <c r="B72" s="25"/>
+      <c r="A72" s="20"/>
+      <c r="B72" s="22"/>
       <c r="C72" s="13"/>
       <c r="D72" s="15"/>
       <c r="E72" s="14"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73" s="23"/>
-      <c r="B73" s="25"/>
+      <c r="A73" s="20"/>
+      <c r="B73" s="22"/>
       <c r="C73" s="13"/>
       <c r="D73" s="15"/>
       <c r="E73" s="14"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A74" s="23"/>
-      <c r="B74" s="25"/>
+      <c r="A74" s="20"/>
+      <c r="B74" s="22"/>
       <c r="C74" s="13"/>
       <c r="D74" s="15"/>
       <c r="E74" s="14"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A75" s="23"/>
-      <c r="B75" s="25"/>
+      <c r="A75" s="20"/>
+      <c r="B75" s="22"/>
       <c r="C75" s="13"/>
       <c r="D75" s="15"/>
       <c r="E75" s="14"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A76" s="23"/>
-      <c r="B76" s="25"/>
+      <c r="A76" s="20"/>
+      <c r="B76" s="22"/>
       <c r="C76" s="13"/>
       <c r="D76" s="15"/>
       <c r="E76" s="14"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77" s="23"/>
-      <c r="B77" s="25"/>
+      <c r="A77" s="20"/>
+      <c r="B77" s="22"/>
       <c r="C77" s="13"/>
       <c r="D77" s="15"/>
       <c r="E77" s="14"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78" s="23"/>
-      <c r="B78" s="25"/>
+      <c r="A78" s="20"/>
+      <c r="B78" s="22"/>
       <c r="C78" s="13"/>
       <c r="D78" s="15"/>
       <c r="E78" s="14"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A79" s="23"/>
-      <c r="B79" s="25"/>
+      <c r="A79" s="20"/>
+      <c r="B79" s="22"/>
       <c r="C79" s="13"/>
       <c r="D79" s="15"/>
       <c r="E79" s="14"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A80" s="23"/>
-      <c r="B80" s="25"/>
+      <c r="A80" s="20"/>
+      <c r="B80" s="22"/>
       <c r="C80" s="13"/>
       <c r="D80" s="15"/>
       <c r="E80" s="14"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A81" s="23"/>
-      <c r="B81" s="25"/>
+      <c r="A81" s="20"/>
+      <c r="B81" s="22"/>
       <c r="C81" s="13"/>
       <c r="D81" s="15"/>
       <c r="E81" s="14"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A82" s="23"/>
-      <c r="B82" s="25"/>
+      <c r="A82" s="20"/>
+      <c r="B82" s="22"/>
       <c r="C82" s="13"/>
       <c r="D82" s="15"/>
       <c r="E82" s="14"/>
     </row>
     <row r="83" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="23"/>
-      <c r="B83" s="25"/>
+      <c r="A83" s="20"/>
+      <c r="B83" s="22"/>
       <c r="C83" s="13"/>
       <c r="D83" s="15"/>
       <c r="E83" s="14"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84" s="23"/>
-      <c r="B84" s="25"/>
+      <c r="A84" s="20"/>
+      <c r="B84" s="22"/>
       <c r="C84" s="13"/>
       <c r="D84" s="15"/>
       <c r="E84" s="14"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A85" s="23"/>
-      <c r="B85" s="25"/>
+      <c r="A85" s="20"/>
+      <c r="B85" s="22"/>
       <c r="C85" s="13"/>
       <c r="D85" s="15"/>
       <c r="E85" s="14"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A86" s="23"/>
-      <c r="B86" s="25"/>
+      <c r="A86" s="20"/>
+      <c r="B86" s="22"/>
       <c r="C86" s="13"/>
       <c r="D86" s="15"/>
       <c r="E86" s="14"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A87" s="23"/>
-      <c r="B87" s="25"/>
+      <c r="A87" s="20"/>
+      <c r="B87" s="22"/>
       <c r="C87" s="13"/>
       <c r="D87" s="15"/>
       <c r="E87" s="14"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88" s="23"/>
-      <c r="B88" s="25"/>
+      <c r="A88" s="20"/>
+      <c r="B88" s="22"/>
       <c r="C88" s="13"/>
       <c r="D88" s="15"/>
       <c r="E88" s="14"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A89" s="23"/>
-      <c r="B89" s="25"/>
+      <c r="A89" s="20"/>
+      <c r="B89" s="22"/>
       <c r="C89" s="13"/>
       <c r="D89" s="15"/>
       <c r="E89" s="14"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="23"/>
-      <c r="B90" s="25"/>
+      <c r="A90" s="20"/>
+      <c r="B90" s="22"/>
       <c r="C90" s="13"/>
       <c r="D90" s="15"/>
       <c r="E90" s="14"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91" s="23"/>
-      <c r="B91" s="25"/>
+      <c r="A91" s="20"/>
+      <c r="B91" s="22"/>
       <c r="C91" s="13"/>
       <c r="D91" s="15"/>
       <c r="E91" s="14"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92" s="23"/>
-      <c r="B92" s="25"/>
+      <c r="A92" s="20"/>
+      <c r="B92" s="22"/>
       <c r="C92" s="13"/>
       <c r="D92" s="15"/>
       <c r="E92" s="14"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93" s="23"/>
-      <c r="B93" s="25"/>
+      <c r="A93" s="20"/>
+      <c r="B93" s="22"/>
       <c r="C93" s="13"/>
       <c r="D93" s="15"/>
       <c r="E93" s="14"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A94" s="23"/>
-      <c r="B94" s="25"/>
+      <c r="A94" s="20"/>
+      <c r="B94" s="22"/>
       <c r="C94" s="13"/>
       <c r="D94" s="15"/>
       <c r="E94" s="14"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="23"/>
-      <c r="B95" s="25"/>
+      <c r="A95" s="20"/>
+      <c r="B95" s="22"/>
       <c r="C95" s="13"/>
       <c r="D95" s="15"/>
       <c r="E95" s="14"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="23"/>
-      <c r="B96" s="25"/>
+      <c r="A96" s="20"/>
+      <c r="B96" s="22"/>
       <c r="C96" s="13"/>
       <c r="D96" s="15"/>
       <c r="E96" s="14"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A97" s="23"/>
-      <c r="B97" s="25"/>
+      <c r="A97" s="20"/>
+      <c r="B97" s="22"/>
       <c r="C97" s="13"/>
       <c r="D97" s="15"/>
       <c r="E97" s="14"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A98" s="23"/>
-      <c r="B98" s="25"/>
+      <c r="A98" s="20"/>
+      <c r="B98" s="22"/>
       <c r="C98" s="13"/>
       <c r="D98" s="15"/>
       <c r="E98" s="14"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="23"/>
-      <c r="B99" s="25"/>
+      <c r="A99" s="20"/>
+      <c r="B99" s="22"/>
       <c r="C99" s="13"/>
       <c r="D99" s="15"/>
       <c r="E99" s="14"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="23"/>
-      <c r="B100" s="25"/>
+      <c r="A100" s="20"/>
+      <c r="B100" s="22"/>
       <c r="C100" s="13"/>
       <c r="D100" s="15"/>
       <c r="E100" s="14"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A101" s="23"/>
-      <c r="B101" s="25"/>
+      <c r="A101" s="20"/>
+      <c r="B101" s="22"/>
       <c r="C101" s="13"/>
       <c r="D101" s="15"/>
       <c r="E101" s="14"/>
     </row>
     <row r="102" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="23"/>
-      <c r="B102" s="25"/>
+      <c r="A102" s="20"/>
+      <c r="B102" s="22"/>
       <c r="C102" s="13"/>
       <c r="D102" s="15"/>
       <c r="E102" s="14"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" s="23"/>
-      <c r="B103" s="25"/>
+      <c r="A103" s="20"/>
+      <c r="B103" s="22"/>
       <c r="C103" s="13"/>
       <c r="D103" s="15"/>
       <c r="E103" s="14"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" s="23"/>
-      <c r="B104" s="25"/>
+      <c r="A104" s="20"/>
+      <c r="B104" s="22"/>
       <c r="C104" s="13"/>
       <c r="D104" s="15"/>
       <c r="E104" s="14"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" s="23"/>
-      <c r="B105" s="25"/>
+      <c r="A105" s="20"/>
+      <c r="B105" s="22"/>
       <c r="C105" s="13"/>
       <c r="D105" s="15"/>
       <c r="E105" s="14"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A106" s="23"/>
-      <c r="B106" s="25"/>
+      <c r="A106" s="20"/>
+      <c r="B106" s="22"/>
       <c r="C106" s="13"/>
       <c r="D106" s="15"/>
       <c r="E106" s="14"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A107" s="23"/>
-      <c r="B107" s="25"/>
+      <c r="A107" s="20"/>
+      <c r="B107" s="22"/>
       <c r="C107" s="13"/>
       <c r="D107" s="15"/>
       <c r="E107" s="14"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A108" s="23"/>
-      <c r="B108" s="25"/>
+      <c r="A108" s="20"/>
+      <c r="B108" s="22"/>
       <c r="C108" s="13"/>
       <c r="D108" s="15"/>
       <c r="E108" s="14"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A109" s="23"/>
-      <c r="B109" s="25"/>
+      <c r="A109" s="20"/>
+      <c r="B109" s="22"/>
       <c r="C109" s="13"/>
       <c r="D109" s="15"/>
       <c r="E109" s="14"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A110" s="23"/>
-      <c r="B110" s="25"/>
+      <c r="A110" s="20"/>
+      <c r="B110" s="22"/>
       <c r="C110" s="13"/>
       <c r="D110" s="15"/>
       <c r="E110" s="14"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A111" s="23"/>
-      <c r="B111" s="25"/>
+      <c r="A111" s="20"/>
+      <c r="B111" s="22"/>
       <c r="C111" s="13"/>
       <c r="D111" s="15"/>
       <c r="E111" s="14"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A112" s="23"/>
-      <c r="B112" s="25"/>
+      <c r="A112" s="20"/>
+      <c r="B112" s="22"/>
       <c r="C112" s="13"/>
       <c r="D112" s="15"/>
       <c r="E112" s="14"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A113" s="23"/>
-      <c r="B113" s="25"/>
+      <c r="A113" s="20"/>
+      <c r="B113" s="22"/>
       <c r="C113" s="13"/>
       <c r="D113" s="15"/>
       <c r="E113" s="14"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A114" s="23"/>
-      <c r="B114" s="25"/>
+      <c r="A114" s="20"/>
+      <c r="B114" s="22"/>
       <c r="C114" s="13"/>
       <c r="D114" s="15"/>
       <c r="E114" s="14"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A115" s="23"/>
-      <c r="B115" s="25"/>
+      <c r="A115" s="20"/>
+      <c r="B115" s="22"/>
       <c r="C115" s="13"/>
       <c r="D115" s="15"/>
       <c r="E115" s="14"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A116" s="23"/>
-      <c r="B116" s="25"/>
+      <c r="A116" s="20"/>
+      <c r="B116" s="22"/>
       <c r="C116" s="13"/>
       <c r="D116" s="15"/>
       <c r="E116" s="14"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A117" s="23"/>
-      <c r="B117" s="25"/>
+      <c r="A117" s="20"/>
+      <c r="B117" s="22"/>
       <c r="C117" s="13"/>
       <c r="D117" s="15"/>
       <c r="E117" s="14"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A118" s="23"/>
-      <c r="B118" s="25"/>
+      <c r="A118" s="20"/>
+      <c r="B118" s="22"/>
       <c r="C118" s="13"/>
       <c r="D118" s="15"/>
       <c r="E118" s="14"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A119" s="23"/>
-      <c r="B119" s="25"/>
+      <c r="A119" s="20"/>
+      <c r="B119" s="22"/>
       <c r="C119" s="13"/>
       <c r="D119" s="15"/>
       <c r="E119" s="14"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A120" s="23"/>
-      <c r="B120" s="25"/>
+      <c r="A120" s="20"/>
+      <c r="B120" s="22"/>
       <c r="C120" s="13"/>
       <c r="D120" s="15"/>
       <c r="E120" s="14"/>
@@ -10373,229 +10373,340 @@
       <c r="B1487" s="11"/>
     </row>
     <row r="1488" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1488" s="32" t="s">
-        <v>159</v>
-      </c>
-      <c r="B1488" s="33"/>
+      <c r="A1488" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1488" s="28"/>
     </row>
     <row r="1489" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1489" s="34"/>
-      <c r="B1489" s="35"/>
+      <c r="A1489" s="29"/>
+      <c r="B1489" s="30"/>
     </row>
     <row r="1490" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1490" s="34"/>
-      <c r="B1490" s="35"/>
+      <c r="A1490" s="29"/>
+      <c r="B1490" s="30"/>
     </row>
     <row r="1491" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1491" s="34"/>
-      <c r="B1491" s="35"/>
+      <c r="A1491" s="29"/>
+      <c r="B1491" s="30"/>
     </row>
     <row r="1492" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1492" s="34"/>
-      <c r="B1492" s="35"/>
+      <c r="A1492" s="29"/>
+      <c r="B1492" s="30"/>
     </row>
     <row r="1493" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1493" s="34"/>
-      <c r="B1493" s="35"/>
+      <c r="A1493" s="29"/>
+      <c r="B1493" s="30"/>
     </row>
     <row r="1494" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1494" s="34"/>
-      <c r="B1494" s="35"/>
+      <c r="A1494" s="29"/>
+      <c r="B1494" s="30"/>
     </row>
     <row r="1495" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1495" s="34"/>
-      <c r="B1495" s="35"/>
+      <c r="A1495" s="29"/>
+      <c r="B1495" s="30"/>
     </row>
     <row r="1496" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1496" s="34"/>
-      <c r="B1496" s="35"/>
+      <c r="A1496" s="29"/>
+      <c r="B1496" s="30"/>
     </row>
     <row r="1497" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1497" s="34"/>
-      <c r="B1497" s="35"/>
+      <c r="A1497" s="29"/>
+      <c r="B1497" s="30"/>
     </row>
     <row r="1498" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1498" s="34"/>
-      <c r="B1498" s="35"/>
+      <c r="A1498" s="29"/>
+      <c r="B1498" s="30"/>
     </row>
     <row r="1499" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1499" s="34"/>
-      <c r="B1499" s="35"/>
+      <c r="A1499" s="29"/>
+      <c r="B1499" s="30"/>
     </row>
     <row r="1500" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1500" s="34"/>
-      <c r="B1500" s="35"/>
+      <c r="A1500" s="29"/>
+      <c r="B1500" s="30"/>
     </row>
     <row r="1501" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1501" s="34"/>
-      <c r="B1501" s="35"/>
+      <c r="A1501" s="29"/>
+      <c r="B1501" s="30"/>
     </row>
     <row r="1502" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1502" s="34"/>
-      <c r="B1502" s="35"/>
+      <c r="A1502" s="29"/>
+      <c r="B1502" s="30"/>
     </row>
     <row r="1503" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1503" s="34"/>
-      <c r="B1503" s="35"/>
+      <c r="A1503" s="29"/>
+      <c r="B1503" s="30"/>
     </row>
     <row r="1504" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1504" s="34"/>
-      <c r="B1504" s="35"/>
+      <c r="A1504" s="29"/>
+      <c r="B1504" s="30"/>
     </row>
     <row r="1505" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1505" s="34"/>
-      <c r="B1505" s="35"/>
+      <c r="A1505" s="29"/>
+      <c r="B1505" s="30"/>
     </row>
     <row r="1506" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1506" s="34"/>
-      <c r="B1506" s="35"/>
+      <c r="A1506" s="29"/>
+      <c r="B1506" s="30"/>
     </row>
     <row r="1507" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1507" s="34"/>
-      <c r="B1507" s="35"/>
+      <c r="A1507" s="29"/>
+      <c r="B1507" s="30"/>
     </row>
     <row r="1508" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1508" s="34"/>
-      <c r="B1508" s="35"/>
+      <c r="A1508" s="29"/>
+      <c r="B1508" s="30"/>
     </row>
     <row r="1509" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1509" s="34"/>
-      <c r="B1509" s="35"/>
+      <c r="A1509" s="29"/>
+      <c r="B1509" s="30"/>
     </row>
     <row r="1510" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1510" s="34"/>
-      <c r="B1510" s="35"/>
+      <c r="A1510" s="29"/>
+      <c r="B1510" s="30"/>
     </row>
     <row r="1511" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1511" s="34"/>
-      <c r="B1511" s="35"/>
+      <c r="A1511" s="29"/>
+      <c r="B1511" s="30"/>
     </row>
     <row r="1512" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1512" s="34"/>
-      <c r="B1512" s="35"/>
+      <c r="A1512" s="29"/>
+      <c r="B1512" s="30"/>
     </row>
     <row r="1513" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1513" s="34"/>
-      <c r="B1513" s="35"/>
+      <c r="A1513" s="29"/>
+      <c r="B1513" s="30"/>
     </row>
     <row r="1514" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1514" s="34"/>
-      <c r="B1514" s="35"/>
+      <c r="A1514" s="29"/>
+      <c r="B1514" s="30"/>
     </row>
     <row r="1515" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1515" s="34"/>
-      <c r="B1515" s="35"/>
+      <c r="A1515" s="29"/>
+      <c r="B1515" s="30"/>
     </row>
     <row r="1516" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1516" s="34"/>
-      <c r="B1516" s="35"/>
+      <c r="A1516" s="29"/>
+      <c r="B1516" s="30"/>
     </row>
     <row r="1517" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1517" s="34"/>
-      <c r="B1517" s="35"/>
+      <c r="A1517" s="29"/>
+      <c r="B1517" s="30"/>
     </row>
     <row r="1518" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1518" s="34"/>
-      <c r="B1518" s="35"/>
+      <c r="A1518" s="29"/>
+      <c r="B1518" s="30"/>
     </row>
     <row r="1519" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1519" s="34"/>
-      <c r="B1519" s="35"/>
+      <c r="A1519" s="29"/>
+      <c r="B1519" s="30"/>
     </row>
     <row r="1520" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1520" s="34"/>
-      <c r="B1520" s="35"/>
+      <c r="A1520" s="29"/>
+      <c r="B1520" s="30"/>
     </row>
     <row r="1521" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1521" s="34"/>
-      <c r="B1521" s="35"/>
+      <c r="A1521" s="29"/>
+      <c r="B1521" s="30"/>
     </row>
     <row r="1522" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1522" s="34"/>
-      <c r="B1522" s="35"/>
+      <c r="A1522" s="29"/>
+      <c r="B1522" s="30"/>
     </row>
     <row r="1523" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1523" s="34"/>
-      <c r="B1523" s="35"/>
+      <c r="A1523" s="29"/>
+      <c r="B1523" s="30"/>
     </row>
     <row r="1524" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1524" s="34"/>
-      <c r="B1524" s="35"/>
+      <c r="A1524" s="29"/>
+      <c r="B1524" s="30"/>
     </row>
     <row r="1525" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1525" s="34"/>
-      <c r="B1525" s="35"/>
+      <c r="A1525" s="29"/>
+      <c r="B1525" s="30"/>
     </row>
     <row r="1526" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1526" s="34"/>
-      <c r="B1526" s="35"/>
+      <c r="A1526" s="29"/>
+      <c r="B1526" s="30"/>
     </row>
     <row r="1527" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1527" s="34"/>
-      <c r="B1527" s="35"/>
+      <c r="A1527" s="29"/>
+      <c r="B1527" s="30"/>
     </row>
     <row r="1528" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1528" s="34"/>
-      <c r="B1528" s="35"/>
+      <c r="A1528" s="29"/>
+      <c r="B1528" s="30"/>
     </row>
     <row r="1529" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1529" s="34"/>
-      <c r="B1529" s="35"/>
+      <c r="A1529" s="29"/>
+      <c r="B1529" s="30"/>
     </row>
     <row r="1530" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1530" s="34"/>
-      <c r="B1530" s="35"/>
+      <c r="A1530" s="29"/>
+      <c r="B1530" s="30"/>
     </row>
     <row r="1531" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1531" s="34"/>
-      <c r="B1531" s="35"/>
+      <c r="A1531" s="29"/>
+      <c r="B1531" s="30"/>
     </row>
     <row r="1532" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1532" s="34"/>
-      <c r="B1532" s="35"/>
+      <c r="A1532" s="29"/>
+      <c r="B1532" s="30"/>
     </row>
     <row r="1533" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1533" s="34"/>
-      <c r="B1533" s="35"/>
+      <c r="A1533" s="29"/>
+      <c r="B1533" s="30"/>
     </row>
     <row r="1534" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1534" s="34"/>
-      <c r="B1534" s="35"/>
+      <c r="A1534" s="29"/>
+      <c r="B1534" s="30"/>
     </row>
     <row r="1535" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1535" s="34"/>
-      <c r="B1535" s="35"/>
+      <c r="A1535" s="29"/>
+      <c r="B1535" s="30"/>
     </row>
     <row r="1536" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1536" s="34"/>
-      <c r="B1536" s="35"/>
+      <c r="A1536" s="29"/>
+      <c r="B1536" s="30"/>
     </row>
     <row r="1537" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1537" s="34"/>
-      <c r="B1537" s="35"/>
+      <c r="A1537" s="29"/>
+      <c r="B1537" s="30"/>
     </row>
     <row r="1538" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1538" s="34"/>
-      <c r="B1538" s="35"/>
+      <c r="A1538" s="29"/>
+      <c r="B1538" s="30"/>
     </row>
     <row r="1539" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1539" s="34"/>
-      <c r="B1539" s="35"/>
+      <c r="A1539" s="29"/>
+      <c r="B1539" s="30"/>
     </row>
     <row r="1540" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1540" s="34"/>
-      <c r="B1540" s="35"/>
+      <c r="A1540" s="29"/>
+      <c r="B1540" s="30"/>
     </row>
     <row r="1541" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1541" s="36"/>
-      <c r="B1541" s="37"/>
+      <c r="A1541" s="31"/>
+      <c r="B1541" s="32"/>
     </row>
     <row r="1542" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1542" s="31"/>
-      <c r="B1542" s="27"/>
+      <c r="A1542" s="23"/>
+      <c r="B1542" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="135">
+    <mergeCell ref="C2:E22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="T12:U12"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="T13:U13"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="T14:U14"/>
+    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="P18:R18"/>
+    <mergeCell ref="T18:U18"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="T19:U19"/>
+    <mergeCell ref="P20:R20"/>
+    <mergeCell ref="T20:U20"/>
+    <mergeCell ref="P15:R15"/>
+    <mergeCell ref="T15:U15"/>
+    <mergeCell ref="P16:R16"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="T17:U17"/>
+    <mergeCell ref="P25:R25"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="T24:U24"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="P21:R21"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="T22:U22"/>
+    <mergeCell ref="P30:R30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="P29:R29"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="T26:U26"/>
+    <mergeCell ref="P27:R27"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="P28:R28"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="P34:R34"/>
+    <mergeCell ref="T34:U34"/>
+    <mergeCell ref="P35:R35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="T31:U31"/>
+    <mergeCell ref="P32:R32"/>
+    <mergeCell ref="T32:U32"/>
+    <mergeCell ref="P33:R33"/>
+    <mergeCell ref="T33:U33"/>
+    <mergeCell ref="P31:R31"/>
+    <mergeCell ref="P39:R39"/>
+    <mergeCell ref="T39:U39"/>
+    <mergeCell ref="P40:R40"/>
+    <mergeCell ref="T40:U40"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="T36:U36"/>
+    <mergeCell ref="P37:R37"/>
+    <mergeCell ref="T37:U37"/>
+    <mergeCell ref="P38:R38"/>
+    <mergeCell ref="T38:U38"/>
+    <mergeCell ref="P46:R46"/>
+    <mergeCell ref="T46:U46"/>
+    <mergeCell ref="P47:R47"/>
+    <mergeCell ref="T47:U47"/>
+    <mergeCell ref="P45:R45"/>
+    <mergeCell ref="T45:U45"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="T44:U44"/>
+    <mergeCell ref="P41:R41"/>
+    <mergeCell ref="T41:U41"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="T42:U42"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="T43:U43"/>
+    <mergeCell ref="P56:R56"/>
+    <mergeCell ref="T56:U56"/>
+    <mergeCell ref="P51:R51"/>
+    <mergeCell ref="T51:U51"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="T52:U52"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="T53:U53"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="T48:U48"/>
+    <mergeCell ref="P49:R49"/>
+    <mergeCell ref="T49:U49"/>
+    <mergeCell ref="P50:R50"/>
+    <mergeCell ref="T50:U50"/>
     <mergeCell ref="C23:E30"/>
     <mergeCell ref="C31:E44"/>
     <mergeCell ref="C45:E63"/>
@@ -10620,117 +10731,6 @@
     <mergeCell ref="T54:U54"/>
     <mergeCell ref="P55:R55"/>
     <mergeCell ref="T55:U55"/>
-    <mergeCell ref="P56:R56"/>
-    <mergeCell ref="T56:U56"/>
-    <mergeCell ref="P51:R51"/>
-    <mergeCell ref="T51:U51"/>
-    <mergeCell ref="P52:R52"/>
-    <mergeCell ref="T52:U52"/>
-    <mergeCell ref="P53:R53"/>
-    <mergeCell ref="T53:U53"/>
-    <mergeCell ref="P48:R48"/>
-    <mergeCell ref="T48:U48"/>
-    <mergeCell ref="P49:R49"/>
-    <mergeCell ref="T49:U49"/>
-    <mergeCell ref="P50:R50"/>
-    <mergeCell ref="T50:U50"/>
-    <mergeCell ref="P46:R46"/>
-    <mergeCell ref="T46:U46"/>
-    <mergeCell ref="P47:R47"/>
-    <mergeCell ref="T47:U47"/>
-    <mergeCell ref="P45:R45"/>
-    <mergeCell ref="T45:U45"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="T44:U44"/>
-    <mergeCell ref="P41:R41"/>
-    <mergeCell ref="T41:U41"/>
-    <mergeCell ref="P42:R42"/>
-    <mergeCell ref="T42:U42"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="T43:U43"/>
-    <mergeCell ref="P39:R39"/>
-    <mergeCell ref="T39:U39"/>
-    <mergeCell ref="P40:R40"/>
-    <mergeCell ref="T40:U40"/>
-    <mergeCell ref="P36:R36"/>
-    <mergeCell ref="T36:U36"/>
-    <mergeCell ref="P37:R37"/>
-    <mergeCell ref="T37:U37"/>
-    <mergeCell ref="P38:R38"/>
-    <mergeCell ref="T38:U38"/>
-    <mergeCell ref="P34:R34"/>
-    <mergeCell ref="T34:U34"/>
-    <mergeCell ref="P35:R35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="T31:U31"/>
-    <mergeCell ref="P32:R32"/>
-    <mergeCell ref="T32:U32"/>
-    <mergeCell ref="P33:R33"/>
-    <mergeCell ref="T33:U33"/>
-    <mergeCell ref="P31:R31"/>
-    <mergeCell ref="P30:R30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="T29:U29"/>
-    <mergeCell ref="P26:R26"/>
-    <mergeCell ref="T26:U26"/>
-    <mergeCell ref="P27:R27"/>
-    <mergeCell ref="T27:U27"/>
-    <mergeCell ref="P28:R28"/>
-    <mergeCell ref="T28:U28"/>
-    <mergeCell ref="P25:R25"/>
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="T24:U24"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="P21:R21"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="T22:U22"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="T19:U19"/>
-    <mergeCell ref="P20:R20"/>
-    <mergeCell ref="T20:U20"/>
-    <mergeCell ref="P15:R15"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="P16:R16"/>
-    <mergeCell ref="T16:U16"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="T17:U17"/>
-    <mergeCell ref="T14:U14"/>
-    <mergeCell ref="P9:R9"/>
-    <mergeCell ref="T9:U9"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="T11:U11"/>
-    <mergeCell ref="P18:R18"/>
-    <mergeCell ref="T18:U18"/>
-    <mergeCell ref="C2:E22"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="T7:U7"/>
-    <mergeCell ref="P5:R5"/>
-    <mergeCell ref="T5:U5"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="T3:U3"/>
-    <mergeCell ref="P4:R4"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="T12:U12"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="T13:U13"/>
-    <mergeCell ref="P14:R14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>